<commit_message>
"Donusturucu" sayfasına "Paralel To Serial Converter" bağlantısı eklendi.
</commit_message>
<xml_diff>
--- a/pages/donusturucu.xlsx
+++ b/pages/donusturucu.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EARGE8PC\Desktop\btk42GithubIo\pages\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Depom\Projects\_GithubIO\pages\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1A263EA-7305-4269-A5C2-318BDE367336}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8196" tabRatio="500"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
   <si>
     <t>Sıra</t>
   </si>
@@ -59,9 +60,6 @@
     <t>Link</t>
   </si>
   <si>
-    <t>CV-PTS-00-000-MCR-P3B0-01</t>
-  </si>
-  <si>
     <t>Parallel To Serial</t>
   </si>
   <si>
@@ -102,12 +100,21 @@
   </si>
   <si>
     <t>https://github.com/btk42/CV-ATB-00-000-MCR-S2B0-01</t>
+  </si>
+  <si>
+    <t>Genel</t>
+  </si>
+  <si>
+    <t>CV-PTS-00-000-000-P3B0-01</t>
+  </si>
+  <si>
+    <t>https://github.com/btk42/CV-PTS-00-000-000-P3B0-01</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -491,7 +498,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K4"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -549,67 +556,69 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>13</v>
-      </c>
       <c r="E2" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="H2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="I2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="J2" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="K2" s="6"/>
+        <v>23</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="3" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="D3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" s="5" t="s">
+      <c r="H3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H3" s="5" t="s">
-        <v>21</v>
-      </c>
       <c r="I3" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="7" t="s">
         <v>24</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -617,40 +626,41 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="K4" s="6"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="K3" r:id="rId1"/>
+    <hyperlink ref="K3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="K2" r:id="rId2" xr:uid="{6A286826-7E58-43E5-9D56-BCA3518DE063}"/>
   </hyperlinks>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
-  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId3"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Sayfa &amp;P</oddFooter>

</xml_diff>